<commit_message>
Semana 6: guion unico con escenas y paso a paso; chequeo de minimo cacheable en la calculadora
</commit_message>
<xml_diff>
--- a/semana-06/calculadora-costos-claude.xlsx
+++ b/semana-06/calculadora-costos-claude.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kevin\Documents\CODERHOUSE\AI AUTOMATION\repos\ai-automation-estudiantes\semana-06\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19F55C3A-425F-469B-8288-7E70C26AB20F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B37D88C6-CE49-49D3-A7F7-FC404F6879ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="81">
   <si>
     <t>Calculadora de costos: API de Claude (Batch y Prompt Caching)</t>
   </si>
@@ -98,6 +98,12 @@
     <t>50% sobre entrada y salida (también sobre el caché).</t>
   </si>
   <si>
+    <t>Mínimo cacheable del modelo (tokens)</t>
+  </si>
+  <si>
+    <t>Si la parte fija es más corta que este mínimo, el caché no se activa. Fuente: hoja Precios.</t>
+  </si>
+  <si>
     <t>2. TOKENS TOTALES</t>
   </si>
   <si>
@@ -110,6 +116,9 @@
     <t>Tokens del prefijo leídos desde caché (todas menos la primera)</t>
   </si>
   <si>
+    <t>¿La parte fija supera el mínimo cacheable? (si dice NO, las filas con caché valen lo mismo que sin caché)</t>
+  </si>
+  <si>
     <t>3. MATRIZ DE COSTOS</t>
   </si>
   <si>
@@ -173,7 +182,7 @@
     <t>NOTAS</t>
   </si>
   <si>
-    <t>- El caché solo funciona si el prefijo supera el mínimo del modelo (hoja Precios). Si es más corto, no da error: simplemente no se guarda y pagás la base.</t>
+    <t>- El caché solo funciona si el prefijo supera el mínimo del modelo (celda B15 y hoja Precios). Si es más corto, no da error: simplemente no se guarda y pagás la base. La planilla lo chequea en la fila 20.</t>
   </si>
   <si>
     <t>- La fila Solo Caching supone que las solicitudes van seguidas (menos de 5 minutos entre una y otra), así el caché se mantiene vivo.</t>
@@ -822,14 +831,25 @@
         <v>24</v>
       </c>
     </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="5">
+        <v>1024</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B17" s="9">
         <f>B4*(B5+B6)</f>
@@ -838,7 +858,7 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B18" s="9">
         <f>B4*B7</f>
@@ -847,44 +867,53 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B19" s="9">
         <f>(B4-1)*B5</f>
         <v>898500</v>
       </c>
     </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B20" s="3" t="str">
+        <f>IF(B5&gt;=B15,"SÍ: el caché aplica","NO: el caché no aplica")</f>
+        <v>SÍ: el caché aplica</v>
+      </c>
+    </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="F22" s="10" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B23" s="12">
         <f>B17/1000000*B9</f>
@@ -907,12 +936,12 @@
         <v>0</v>
       </c>
       <c r="G23" s="14" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="15" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B24" s="12">
         <f>B23*(1-$B$14)</f>
@@ -935,15 +964,15 @@
         <v>0.5</v>
       </c>
       <c r="G24" s="14" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="15" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B25" s="12">
-        <f>B5/1000000*B11+B19/1000000*B13+B4*B6/1000000*B9</f>
+        <f>IF($B$5&gt;=$B$15,B5/1000000*B11+B19/1000000*B13+B4*B6/1000000*B9,B23)</f>
         <v>0.54344999999999999</v>
       </c>
       <c r="C25" s="12">
@@ -963,15 +992,15 @@
         <v>0.52828431372549023</v>
       </c>
       <c r="G25" s="14" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="15" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B26" s="12">
-        <f>(B5/1000000*B12+B19/1000000*B13+B4*B6/1000000*B9)*(1-$B$14)</f>
+        <f>IF($B$5&gt;=$B$15,(B5/1000000*B12+B19/1000000*B13+B4*B6/1000000*B9)*(1-$B$14),B24)</f>
         <v>0.27284999999999998</v>
       </c>
       <c r="C26" s="12">
@@ -991,17 +1020,17 @@
         <v>0.7637745098039217</v>
       </c>
       <c r="G26" s="14" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B29" s="16">
         <f>B4*B5/1000000*B9</f>
@@ -1010,16 +1039,16 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B30" s="16">
-        <f>B5/1000000*B11+B19/1000000*B13</f>
+        <f>IF(B5&gt;=B15,B5/1000000*B11+B19/1000000*B13,B29)</f>
         <v>0.18345</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B31" s="17">
         <f>IF(B29=0,0,(B29-B30)/B29)</f>
@@ -1028,32 +1057,32 @@
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -1077,52 +1106,52 @@
   <sheetData>
     <row r="1" spans="1:11" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B5" s="12">
         <v>1</v>
@@ -1152,7 +1181,7 @@
         <v>200000</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -1187,12 +1216,12 @@
         <v>1000000</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B7" s="12">
         <v>5</v>
@@ -1222,32 +1251,32 @@
         <v>1000000</v>
       </c>
       <c r="K7" s="15" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Semana 6: tokens medidos en el Playground y matriz de costos actualizada
</commit_message>
<xml_diff>
--- a/semana-06/calculadora-costos-claude.xlsx
+++ b/semana-06/calculadora-costos-claude.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kevin\Documents\CODERHOUSE\AI AUTOMATION\repos\ai-automation-estudiantes\semana-06\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B37D88C6-CE49-49D3-A7F7-FC404F6879ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33EEE414-EC4B-4615-8EAC-32A3583AAB43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
     <t>Calculadora de costos: API de Claude (Batch y Prompt Caching)</t>
   </si>
   <si>
-    <t>Editá SOLO las celdas amarillas con texto azul. Todo lo demás se calcula solo. Ejemplo cargado: reporte mensual de Agencia Norte con Claude Sonnet 5.</t>
+    <t>Editá SOLO las celdas amarillas con texto azul. Todo lo demás se calcula solo. Ejemplo cargado: reporte mensual de Agencia Norte con Claude Sonnet 5 (tokens medidos en el Playground de Claude el 28/09/2026).</t>
   </si>
   <si>
     <t>1. SUPUESTOS DE TU CASO</t>
@@ -41,19 +41,19 @@
     <t>Tokens de la parte FIJA (prefijo) por solicitud</t>
   </si>
   <si>
-    <t>Estimado para la plantilla de la Guía 1. El número exacto lo muestra el Playground de Claude.</t>
+    <t>Medido en el Playground de Claude con Sonnet 5: entrada con el mensaje 'Hola' (2.264) menos 3.</t>
   </si>
   <si>
     <t>Tokens de la parte VARIABLE por solicitud</t>
   </si>
   <si>
-    <t>Un correo de consulta típico, con remitente y fecha.</t>
+    <t>Medido: promedio de Martina (212) y Julián (142) = entrada de cada uno menos la parte fija.</t>
   </si>
   <si>
     <t>Tokens de SALIDA por solicitud (respuesta)</t>
   </si>
   <si>
-    <t>El JSON con razonamiento, servicio, presupuesto, prioridad y resumen.</t>
+    <t>Medido: promedio de las respuestas de Martina (144) y Julián (126).</t>
   </si>
   <si>
     <t>Modelo elegido</t>
@@ -726,7 +726,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="5">
-        <v>1500</v>
+        <v>2261</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>6</v>
@@ -737,7 +737,7 @@
         <v>7</v>
       </c>
       <c r="B6" s="5">
-        <v>300</v>
+        <v>177</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>8</v>
@@ -748,7 +748,7 @@
         <v>9</v>
       </c>
       <c r="B7" s="5">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>10</v>
@@ -853,7 +853,7 @@
       </c>
       <c r="B17" s="9">
         <f>B4*(B5+B6)</f>
-        <v>1080000</v>
+        <v>1462800</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -862,7 +862,7 @@
       </c>
       <c r="B18" s="9">
         <f>B4*B7</f>
-        <v>90000</v>
+        <v>81000</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -871,7 +871,7 @@
       </c>
       <c r="B19" s="9">
         <f>(B4-1)*B5</f>
-        <v>898500</v>
+        <v>1354339</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -917,15 +917,15 @@
       </c>
       <c r="B23" s="12">
         <f>B17/1000000*B9</f>
-        <v>2.16</v>
+        <v>2.9256000000000002</v>
       </c>
       <c r="C23" s="12">
         <f>B18/1000000*B10</f>
-        <v>0.89999999999999991</v>
+        <v>0.81</v>
       </c>
       <c r="D23" s="12">
         <f>B23+C23</f>
-        <v>3.06</v>
+        <v>3.7356000000000003</v>
       </c>
       <c r="E23" s="12">
         <f>$D$23-D23</f>
@@ -945,19 +945,19 @@
       </c>
       <c r="B24" s="12">
         <f>B23*(1-$B$14)</f>
-        <v>1.08</v>
+        <v>1.4628000000000001</v>
       </c>
       <c r="C24" s="12">
         <f>C23*(1-$B$14)</f>
-        <v>0.44999999999999996</v>
+        <v>0.40500000000000003</v>
       </c>
       <c r="D24" s="12">
         <f>B24+C24</f>
-        <v>1.53</v>
+        <v>1.8678000000000001</v>
       </c>
       <c r="E24" s="12">
         <f>$D$23-D24</f>
-        <v>1.53</v>
+        <v>1.8678000000000001</v>
       </c>
       <c r="F24" s="13">
         <f>IF($D$23=0,0,E24/$D$23)</f>
@@ -973,23 +973,23 @@
       </c>
       <c r="B25" s="12">
         <f>IF($B$5&gt;=$B$15,B5/1000000*B11+B19/1000000*B13+B4*B6/1000000*B9,B23)</f>
-        <v>0.54344999999999999</v>
+        <v>0.48892029999999997</v>
       </c>
       <c r="C25" s="12">
         <f>C23</f>
-        <v>0.89999999999999991</v>
+        <v>0.81</v>
       </c>
       <c r="D25" s="12">
         <f>B25+C25</f>
-        <v>1.4434499999999999</v>
+        <v>1.2989203</v>
       </c>
       <c r="E25" s="12">
         <f>$D$23-D25</f>
-        <v>1.6165500000000002</v>
+        <v>2.4366797</v>
       </c>
       <c r="F25" s="13">
         <f>IF($D$23=0,0,E25/$D$23)</f>
-        <v>0.52828431372549023</v>
+        <v>0.65228603169504229</v>
       </c>
       <c r="G25" s="14" t="s">
         <v>45</v>
@@ -1001,23 +1001,23 @@
       </c>
       <c r="B26" s="12">
         <f>IF($B$5&gt;=$B$15,(B5/1000000*B12+B19/1000000*B13+B4*B6/1000000*B9)*(1-$B$14),B24)</f>
-        <v>0.27284999999999998</v>
+        <v>0.24615589999999998</v>
       </c>
       <c r="C26" s="12">
         <f>C23*(1-$B$14)</f>
-        <v>0.44999999999999996</v>
+        <v>0.40500000000000003</v>
       </c>
       <c r="D26" s="12">
         <f>B26+C26</f>
-        <v>0.72284999999999999</v>
+        <v>0.65115590000000001</v>
       </c>
       <c r="E26" s="12">
         <f>$D$23-D26</f>
-        <v>2.3371500000000003</v>
+        <v>3.0844441000000002</v>
       </c>
       <c r="F26" s="13">
         <f>IF($D$23=0,0,E26/$D$23)</f>
-        <v>0.7637745098039217</v>
+        <v>0.82568907270585712</v>
       </c>
       <c r="G26" s="14" t="s">
         <v>47</v>
@@ -1034,7 +1034,7 @@
       </c>
       <c r="B29" s="16">
         <f>B4*B5/1000000*B9</f>
-        <v>1.8</v>
+        <v>2.7132000000000001</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="B30" s="16">
         <f>IF(B5&gt;=B15,B5/1000000*B11+B19/1000000*B13,B29)</f>
-        <v>0.18345</v>
+        <v>0.2765203</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>